<commit_message>
Update API routes for renamed schema
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/api-spec.xlsx
+++ b/docs/api-spec.xlsx
@@ -700,7 +700,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="42" customWidth="1"/>
+    <col min="1" max="1" width="46" customWidth="1"/>
     <col min="2" max="2" width="46" customWidth="1"/>
     <col min="3" max="3" width="46" customWidth="1"/>
   </cols>
@@ -1215,7 +1215,7 @@
     <row r="60">
       <c r="A60" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">定義と違うメソッド (POST /api/employees)</t>
+          <t xml:space="preserve">定義と違うメソッド (POST /api/people)</t>
         </is>
       </c>
       <c r="B60" s="9">
@@ -1230,12 +1230,12 @@
     <row r="61">
       <c r="A61" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">末尾スラッシュ付き (GET /api/duties/)</t>
+          <t xml:space="preserve">末尾スラッシュ付き (GET /api/lottery-results/)</t>
         </is>
       </c>
       <c r="B61" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">301 で /api/duties へリダイレクト</t>
+          <t xml:space="preserve">301 で /api/lottery-results へリダイレクト</t>
         </is>
       </c>
       <c r="C61" s="8" t="inlineStr">
@@ -1263,8 +1263,8 @@
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="2" width="8" customWidth="1"/>
-    <col min="3" max="3" width="32" customWidth="1"/>
-    <col min="4" max="4" width="29" customWidth="1"/>
+    <col min="3" max="3" width="41" customWidth="1"/>
+    <col min="4" max="4" width="33" customWidth="1"/>
     <col min="5" max="5" width="8" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1339,7 +1339,7 @@
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">/api/employees</t>
+          <t xml:space="preserve">/api/people</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
@@ -1364,12 +1364,12 @@
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">/api/areas</t>
+          <t xml:space="preserve">/api/tasks</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">掃除エリア一覧</t>
+          <t xml:space="preserve">掃除タスク一覧</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
@@ -1389,12 +1389,12 @@
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">/api/duties</t>
+          <t xml:space="preserve">/api/lottery-results</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">当番一覧</t>
+          <t xml:space="preserve">抽選結果一覧</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
@@ -1414,12 +1414,12 @@
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">/api/duties/generate</t>
+          <t xml:space="preserve">/api/lottery-results/generate</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">翌週分の当番を生成</t>
+          <t xml:space="preserve">翌週分の抽選結果を生成</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
@@ -1439,12 +1439,12 @@
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">/api/duties/{id}</t>
+          <t xml:space="preserve">/api/lottery-results/{id}</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">当番の状態を更新 (完了報告)</t>
+          <t xml:space="preserve">抽選結果の状態を更新 (完了報告)</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
@@ -1464,12 +1464,12 @@
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">/api/duties/{id}/swap-requests</t>
+          <t xml:space="preserve">/api/lottery-results/{id}/skip-requests</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">交代申請の作成</t>
+          <t xml:space="preserve">スキップ申請の作成</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
@@ -1489,12 +1489,12 @@
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">/api/swap-requests/{id}</t>
+          <t xml:space="preserve">/api/skip-requests/{id}</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">交代申請の承認・却下</t>
+          <t xml:space="preserve">スキップ申請の承認・却下</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
@@ -2370,7 +2370,7 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">5.2 GET /api/employees</t>
+          <t xml:space="preserve">5.2 GET /api/people</t>
         </is>
       </c>
     </row>
@@ -2500,7 +2500,7 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">curl http://localhost:8080/api/employees</t>
+          <t xml:space="preserve">curl http://localhost:8080/api/people</t>
         </is>
       </c>
     </row>
@@ -2516,7 +2516,7 @@
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">5.3 GET /api/areas</t>
+          <t xml:space="preserve">5.3 GET /api/tasks</t>
         </is>
       </c>
     </row>
@@ -2627,7 +2627,7 @@
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">curl http://localhost:8080/api/areas</t>
+          <t xml:space="preserve">curl http://localhost:8080/api/tasks</t>
         </is>
       </c>
     </row>
@@ -2635,7 +2635,7 @@
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">5.4 GET /api/duties</t>
+          <t xml:space="preserve">5.4 GET /api/lottery-results</t>
         </is>
       </c>
     </row>
@@ -2814,7 +2814,7 @@
     <row r="98">
       <c r="A98" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">curl http://localhost:8080/api/duties</t>
+          <t xml:space="preserve">curl http://localhost:8080/api/lottery-results</t>
         </is>
       </c>
     </row>
@@ -2852,7 +2852,7 @@
     <row r="106">
       <c r="A106" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">5.5 POST /api/duties/generate</t>
+          <t xml:space="preserve">5.5 POST /api/lottery-results/generate</t>
         </is>
       </c>
     </row>
@@ -3036,7 +3036,7 @@
     <row r="133">
       <c r="A133" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">curl -X POST http://localhost:8080/api/duties/generate</t>
+          <t xml:space="preserve">curl -X POST http://localhost:8080/api/lottery-results/generate</t>
         </is>
       </c>
     </row>
@@ -3160,21 +3160,21 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">curl http://localhost:8080/api/employees</t>
+          <t xml:space="preserve">curl http://localhost:8080/api/people</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">curl http://localhost:8080/api/areas</t>
+          <t xml:space="preserve">curl http://localhost:8080/api/tasks</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">curl http://localhost:8080/api/duties</t>
+          <t xml:space="preserve">curl http://localhost:8080/api/lottery-results</t>
         </is>
       </c>
     </row>
@@ -3191,7 +3191,7 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">curl -X POST http://localhost:8080/api/duties/generate</t>
+          <t xml:space="preserve">curl -X POST http://localhost:8080/api/lottery-results/generate</t>
         </is>
       </c>
     </row>
@@ -3208,7 +3208,7 @@
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">curl -s http://localhost:8080/api/duties | python3 -m json.tool</t>
+          <t xml:space="preserve">curl -s http://localhost:8080/api/lottery-results | python3 -m json.tool</t>
         </is>
       </c>
     </row>
@@ -3224,14 +3224,14 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Invoke-RestMethod http://localhost:8080/api/duties</t>
+          <t xml:space="preserve">Invoke-RestMethod http://localhost:8080/api/lottery-results</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Invoke-RestMethod -Method Post http://localhost:8080/api/duties/generate</t>
+          <t xml:space="preserve">Invoke-RestMethod -Method Post http://localhost:8080/api/lottery-results/generate</t>
         </is>
       </c>
     </row>
@@ -3270,7 +3270,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">7.1 PATCH /api/duties/{id} — 当番の状態更新</t>
+          <t xml:space="preserve">7.1 PATCH /api/lottery-results/{id} — 抽選結果の状態更新</t>
         </is>
       </c>
     </row>
@@ -3553,7 +3553,7 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">7.2 POST /api/duties/{id}/swap-requests — 交代申請の作成</t>
+          <t xml:space="preserve">7.2 POST /api/lottery-results/{id}/skip-requests — スキップ申請の作成</t>
         </is>
       </c>
     </row>
@@ -3807,7 +3807,7 @@
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">7.3 PATCH /api/swap-requests/{id} — 交代申請の承認・却下</t>
+          <t xml:space="preserve">7.3 PATCH /api/skip-requests/{id} — スキップ申請の承認・却下</t>
         </is>
       </c>
     </row>
@@ -3983,7 +3983,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
-    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="2" max="2" width="26" customWidth="1"/>
     <col min="3" max="3" width="39" customWidth="1"/>
     <col min="4" max="4" width="46" customWidth="1"/>
   </cols>
@@ -4044,7 +4044,7 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">「自分の当番」の取得</t>
+          <t xml:space="preserve">「自分の抽選結果」の取得</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
@@ -4054,7 +4054,7 @@
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">認証と合わせて決める。GET /api/duties/me を作るか</t>
+          <t xml:space="preserve">認証と合わせて決める。GET /api/lottery-results/me を作るか</t>
         </is>
       </c>
     </row>

</xml_diff>